<commit_message>
fixed bugs and updated input
</commit_message>
<xml_diff>
--- a/config_data/units_mapping.xlsx
+++ b/config_data/units_mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\output_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9145" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9147" uniqueCount="353">
   <si>
     <t>Resource Name</t>
   </si>
@@ -1077,6 +1077,9 @@
   </si>
   <si>
     <t>Desired_unit</t>
+  </si>
+  <si>
+    <t>km/(vehicle*a)</t>
   </si>
 </sst>
 </file>
@@ -34870,10 +34873,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -35044,6 +35047,14 @@
         <v>19</v>
       </c>
     </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>352</v>
+      </c>
+      <c r="B22" t="s">
+        <v>352</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
corrected unit conversion for non group processes
</commit_message>
<xml_diff>
--- a/config_data/units_mapping.xlsx
+++ b/config_data/units_mapping.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65E7D8D-7910-4BC0-A822-C7122756C556}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Unique Units" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -99,9 +100,6 @@
     <t>MEUR/vehicle</t>
   </si>
   <si>
-    <t>MEUR/pkm</t>
-  </si>
-  <si>
     <t>Bpkm</t>
   </si>
   <si>
@@ -121,12 +119,15 @@
   </si>
   <si>
     <t>MEUR/GW</t>
+  </si>
+  <si>
+    <t>MEUR/Bpkm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -174,7 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -473,24 +474,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -498,7 +499,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -506,7 +507,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -514,15 +515,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -530,7 +531,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -538,7 +539,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -546,23 +547,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>27</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -570,7 +571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -578,7 +579,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -586,7 +587,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -594,7 +595,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -602,7 +603,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -610,7 +611,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -618,7 +619,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -626,7 +627,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -634,7 +635,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -642,28 +643,28 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>30</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>31</v>
       </c>
-      <c r="B23" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>32</v>
-      </c>
-      <c r="B24" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added process grp unit conversion
</commit_message>
<xml_diff>
--- a/config_data/units_mapping.xlsx
+++ b/config_data/units_mapping.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t>Unit</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>GW</t>
-  </si>
-  <si>
-    <t>Km/a</t>
   </si>
   <si>
     <t>GW/GW</t>
@@ -493,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -501,7 +498,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -525,7 +522,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -554,18 +551,18 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +578,7 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -605,15 +602,15 @@
         <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
         <v>34</v>
-      </c>
-      <c r="B16" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -621,7 +618,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -658,26 +655,26 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" t="s">
         <v>31</v>
-      </c>
-      <c r="B24" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update data and add unit conversion for emission factors
</commit_message>
<xml_diff>
--- a/config_data/units_mapping.xlsx
+++ b/config_data/units_mapping.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="36">
   <si>
     <t>Unit</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>GWh</t>
+  </si>
+  <si>
+    <t>g/GJ</t>
   </si>
 </sst>
 </file>
@@ -477,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -677,6 +680,14 @@
         <v>31</v>
       </c>
     </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>